<commit_message>
Add input Users portabilidad
</commit_message>
<xml_diff>
--- a/storage/app/public/UpdatePersonal.xlsx
+++ b/storage/app/public/UpdatePersonal.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Hoja1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Hoja1!$A$1:$AZ$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Hoja1!$A$1:$BA$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t xml:space="preserve">cod_profit</t>
   </si>
@@ -166,6 +166,9 @@
     <t xml:space="preserve">skill</t>
   </si>
   <si>
+    <t xml:space="preserve">usuario_crm_portabilidad</t>
+  </si>
+  <si>
     <t xml:space="preserve">contrato1</t>
   </si>
   <si>
@@ -185,32 +188,16 @@
   </si>
   <si>
     <t xml:space="preserve">porcentajes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">estatus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fecha_egreso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motivo_egreso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Egresado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Renuncia</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="@"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -360,15 +347,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -580,7 +567,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:BE1048576"/>
+  <dimension ref="A1:BF1048576"/>
   <sheetFormatPr defaultColWidth="10.14453125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.43"/>
@@ -621,18 +608,19 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="44" min="44" style="1" width="23.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="45" min="45" style="1" width="34.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="47" min="46" style="1" width="15.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="13.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="51" min="49" style="1" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="52" style="1" width="14.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="2" width="16.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="2" width="13.43"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="55" min="55" style="2" width="10.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="56" min="56" style="2" width="12.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="57" min="57" style="2" width="13.69"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="58" style="2" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="48" min="48" style="1" width="24.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="49" min="49" style="1" width="13.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="52" min="50" style="1" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="53" min="53" style="1" width="14.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="54" min="54" style="2" width="16.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="55" min="55" style="2" width="13.43"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="56" min="56" style="2" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="57" min="57" style="2" width="12.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="58" min="58" style="2" width="13.69"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="59" style="2" width="10.14"/>
   </cols>
   <sheetData>
-    <row r="1" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" s="9" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -777,10 +765,10 @@
       <c r="AV1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="AW1" s="6" t="s">
+      <c r="AW1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="AX1" s="3" t="s">
+      <c r="AX1" s="6" t="s">
         <v>49</v>
       </c>
       <c r="AY1" s="3" t="s">
@@ -789,36 +777,27 @@
       <c r="AZ1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="BA1" s="7" t="s">
+      <c r="BA1" s="3" t="s">
         <v>52</v>
       </c>
       <c r="BB1" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="8" t="s">
+      <c r="BC1" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="BE1" s="8" t="s">
-        <v>56</v>
-      </c>
+      <c r="BD1" s="8"/>
+      <c r="BE1" s="8"/>
+      <c r="BF1" s="8"/>
     </row>
-    <row r="2" s="8" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C2" s="8" t="n">
+    <row r="2" s="9" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C2" s="9" t="n">
         <v>19754617</v>
       </c>
-      <c r="AV2" s="9"/>
-      <c r="BC2" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="BD2" s="10" t="n">
-        <v>46163</v>
-      </c>
-      <c r="BE2" s="8" t="s">
-        <v>58</v>
-      </c>
+      <c r="AW2" s="10"/>
+      <c r="BD2" s="8"/>
+      <c r="BE2" s="8"/>
+      <c r="BF2" s="8"/>
     </row>
     <row r="1048530" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1048531" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>